<commit_message>
feat: add dataset alignment script and generate updated excel and documentation trackers
</commit_message>
<xml_diff>
--- a/compitiations/Ally_Vision_Competitions_Master_Tracker.xlsx
+++ b/compitiations/Ally_Vision_Competitions_Master_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ECU\GraduationProject\compitiations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{190A69ED-CD2F-4568-95E5-8CFB5D1C15E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849FC276-F5FB-4902-8E26-80936AA4F64C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2314,7 +2314,7 @@
       <c r="C10" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="31" t="s">
         <v>61</v>
       </c>
       <c r="E10" s="11" t="s">
@@ -2710,7 +2710,7 @@
       <c r="C21" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="32" t="s">
         <v>144</v>
       </c>
       <c r="E21" s="5" t="s">
@@ -2746,7 +2746,7 @@
       <c r="C22" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="31" t="s">
         <v>152</v>
       </c>
       <c r="E22" s="11" t="s">
@@ -2998,7 +2998,7 @@
       <c r="C29" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="32" t="s">
         <v>77</v>
       </c>
       <c r="E29" s="5" t="s">
@@ -3034,7 +3034,7 @@
       <c r="C30" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="31" t="s">
         <v>77</v>
       </c>
       <c r="E30" s="11" t="s">

</xml_diff>